<commit_message>
Regenerate TCB after merging CI auto-analysis, using the new Beta/Rf cache fallback
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026_07_03.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026_07_03.xlsx
@@ -15200,14 +15200,14 @@
     <row r="3">
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Ngân hàng TCB</t>
+          <t>Ngân hàng Thương mại Cổ phần Kỹ thương Việt Nam</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Ngày lập: 03/07/2026 16:31</t>
+          <t>Ngày lập: 03/07/2026 16:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Rf (risk-free rate) fetch: both prior sources had broken externally
worldgovernmentbonds.com now renders the yield via client-side JavaScript (a requests-based
scrape can't see it), and Vietcap's bond-yield API endpoint now 404s (moved/renamed) - neither
is related to GitHub Actions or IP blocking, both sites changed independently over time. Added
investing.com (via the existing curl TLS-fingerprint-bypass trick already used elsewhere) as the
new primary source, confirmed working (4.53% live vs the 4.50% hardcoded fallback). Kept the two
old sources as secondary attempts in case they get fixed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026_07_03.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026_07_03.xlsx
@@ -12408,19 +12408,19 @@
         <v>0.08</v>
       </c>
       <c r="B3" s="19" t="n">
-        <v>43564.68451431155</v>
+        <v>43404.13391176899</v>
       </c>
       <c r="C3" s="19" t="n">
-        <v>46371.48321761995</v>
+        <v>46186.93046986223</v>
       </c>
       <c r="D3" s="19" t="n">
-        <v>50301.0014022517</v>
+        <v>50082.84565119277</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>56195.27867919933</v>
+        <v>55926.71842318856</v>
       </c>
       <c r="F3" s="19" t="n">
-        <v>66019.07414077871</v>
+        <v>65666.50637651491</v>
       </c>
     </row>
     <row r="4">
@@ -12428,19 +12428,19 @@
         <v>0.1</v>
       </c>
       <c r="B4" s="19" t="n">
-        <v>39308.31058359002</v>
+        <v>39184.25245362469</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>40886.61292882228</v>
+        <v>40749.05805538224</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>42915.85880126376</v>
+        <v>42760.95097192767</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>45621.51996451905</v>
+        <v>45443.4748606549</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>49409.44559307647</v>
+        <v>49199.00830487303</v>
       </c>
     </row>
     <row r="5">
@@ -12448,19 +12448,19 @@
         <v>0.12</v>
       </c>
       <c r="B5" s="19" t="n">
-        <v>36607.02295738964</v>
+        <v>36506.15535580037</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>37603.52762689216</v>
+        <v>37494.13848446107</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>38821.47777850633</v>
+        <v>38701.67341949082</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>40343.91546802406</v>
+        <v>40211.092088278</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>42301.33535454684</v>
+        <v>42151.77323386152</v>
       </c>
     </row>
     <row r="6">
@@ -12468,19 +12468,19 @@
         <v>0.14</v>
       </c>
       <c r="B6" s="19" t="n">
-        <v>34742.70514036096</v>
+        <v>34657.86726154733</v>
       </c>
       <c r="C6" s="29" t="n">
-        <v>35420.93009871419</v>
+        <v>35330.2924260216</v>
       </c>
       <c r="D6" s="29" t="n">
-        <v>36222.46868585892</v>
+        <v>36124.97671130936</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>37184.31499043259</v>
+        <v>37078.59785365468</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>38359.90491824486</v>
+        <v>38244.13480541008</v>
       </c>
     </row>
     <row r="7">
@@ -12488,19 +12488,19 @@
         <v>0.16</v>
       </c>
       <c r="B7" s="19" t="n">
-        <v>33380.26251826892</v>
+        <v>33307.15929398456</v>
       </c>
       <c r="C7" s="29" t="n">
-        <v>33866.86329227887</v>
+        <v>33789.59893509038</v>
       </c>
       <c r="D7" s="29" t="n">
-        <v>34428.32572382881</v>
+        <v>34346.26005944324</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>35083.36522730373</v>
+        <v>34995.69803785493</v>
       </c>
       <c r="F7" s="19" t="n">
-        <v>35857.50282231955</v>
+        <v>35763.2156487051</v>
       </c>
     </row>
   </sheetData>
@@ -14464,7 +14464,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0.045</v>
+        <v>0.04534</v>
       </c>
     </row>
     <row r="5">
@@ -15207,7 +15207,7 @@
     <row r="4">
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Ngày lập: 03/07/2026 16:44</t>
+          <t>Ngày lập: 03/07/2026 17:34</t>
         </is>
       </c>
     </row>
@@ -15653,13 +15653,13 @@
       <c r="E12" s="14" t="n"/>
       <c r="F12" s="14" t="n"/>
       <c r="G12" s="16" t="n">
-        <v>0.140152</v>
+        <v>0.140492</v>
       </c>
       <c r="H12" s="16" t="n">
-        <v>0.140152</v>
+        <v>0.140492</v>
       </c>
       <c r="I12" s="16" t="n">
-        <v>0.140152</v>
+        <v>0.140492</v>
       </c>
     </row>
     <row r="13">

</xml_diff>